<commit_message>
Fixed link to video.
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Dropbox/SPS Dropbox/Jason Bryer/Teaching/DATA606 2026 Spring/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonbryer/SPS Dropbox/Jason Bryer/Teaching/DATA606 2026 Spring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E58DEE-4647-F34A-917A-D1E5B921618D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D2E4BDD-9128-3C4A-A852-FCE2E6C16731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="11540" windowWidth="28760" windowHeight="16060" xr2:uid="{A772458D-4E7B-8249-8B6B-34FE7D5BD316}"/>
+    <workbookView xWindow="1480" yWindow="3580" windowWidth="28760" windowHeight="16060" xr2:uid="{A772458D-4E7B-8249-8B6B-34FE7D5BD316}"/>
   </bookViews>
   <sheets>
     <sheet name="Meetups" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
     <t>00-Intro_to_Course</t>
   </si>
   <si>
-    <t>LLcSKd7aSJU</t>
+    <t>H2Lrb8nt3CU</t>
   </si>
 </sst>
 </file>

</xml_diff>